<commit_message>
Daily job scrape update
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -909,35 +909,35 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>ProGlove</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>Senior Technical Project Manager</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" t="n">
         <v>6</v>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Munich Office</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>https://proglove.jobs.personio.de/job/2732130</t>
         </is>

</xml_diff>